<commit_message>
Devolver la ficha de la rutina a Instrucciones!B6:B9
El cargador de Rutinas PRO exige Instrucciones!B3 y B6:B9 con contenido,
y al reconstruir los libros la ficha había quedado a partir de la fila 27,
por lo que la app rechazaba los 63 Excel ("Ningún Excel publicado es
válido").

Ahora la hoja Instrucciones queda así:
- B3: sistema de progresión.
- B6:B9: Rutina generada, Objetivo, Notas de diseño y Progresión
  recomendada, las cuatro siempre rellenas (en las rutinas 1-5 el antiguo
  campo RIR pasa a Notas de diseño).
- Debajo, los campos extra (Gestión de esfuerzo, Intensificadores) y el
  texto de uso de la plantilla de la app.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L2iVMugX1fVtKKv64JLu4m
</commit_message>
<xml_diff>
--- a/EN/rutina_10_2_dias_hombre_mev_60min.xlsx
+++ b/EN/rutina_10_2_dias_hombre_mev_60min.xlsx
@@ -412,11 +412,12 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="1" t="str">
-        <x:v>PLANTILLA DE ENTRENAMIENTO · TRUELIFT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2"/>
+      <x:c r="A1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PLANTILLA DE ENTRENAMIENTO · TRUELIFT</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="inlineStr">
         <x:is>
@@ -429,212 +430,203 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="4"/>
-    <x:row r="5"/>
     <x:row r="6">
-      <x:c r="A6" t="inlineStr">
+      <x:c r="A6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Rutina generada:</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B6" s="0" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Routine 10 - 2 days - MEV hypertrophy, 60 min max - men</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Objetivo:</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" s="0" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">General hypertrophy with minimum effective volume, sessions under 60 minutes, and exercises with quick setup.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Notas de diseño:</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" s="0" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Machines, cables, and stable movement patterns are prioritized to reduce specific warm-ups, equipment changes, and nonproductive fatigue.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Progresión recomendada:</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B9" s="0" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Double progression: when all sets reach the top of the range at the prescribed RIR, increase the load by the smallest possible amount and return to the bottom of the range.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Intensificadores:</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B10" s="0" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Superset = alternate the sets of the two linked exercises with no rest between them; drop set = after the last set, successive load drops with no rest. Each row allows only one method (top+back, superset or drop set). Day 1: superset Press en máquina convergente + Remo en máquina con apoyo de pecho; superset Extensión en cuerda en polea + Curl en cuerda en polea; drop set Elevación lateral en máquina (-20 %). Day 2: superset Press inclinado en máquina + Jalón al pecho agarre neutro cerrado; superset Gemelo en prensa + Crunch en máquina; drop set Curl femoral tumbado (-20 %).</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Cómo usar esta plantilla (rellénala en Excel o LibreOffice):</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="inlineStr">
+    <x:row r="13">
+      <x:c r="A13" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1) Elige arriba el sistema: "simple" o "doble".</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="inlineStr">
+    <x:row r="14">
+      <x:c r="A14" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2) En cada pestaña Día 1..Día 5: nombre de la sesión (B1) y ejercicios.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="inlineStr">
+    <x:row r="15">
+      <x:c r="A15" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">3) Elige PATRÓN (A) y, según el patrón, el EJERCICIO (B).</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="inlineStr">
+    <x:row r="16">
+      <x:c r="A16" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">   Indica SERIES, RIR objetivo y repeticiones.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="inlineStr">
+    <x:row r="17">
+      <x:c r="A17" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">   - SIMPLE: solo "Reps mín / objetivo".</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="inlineStr">
+    <x:row r="18">
+      <x:c r="A18" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">   - DOBLE: "Reps mín" y "Reps máx".</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="inlineStr">
+    <x:row r="19">
+      <x:c r="A19" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">4) DESCANSO (min): admite medios minutos (0,5).</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="inlineStr">
+    <x:row r="20">
+      <x:c r="A20" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">5) Deja el PATRÓN en "(Ninguno)" en las filas que no uses.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="inlineStr">
+    <x:row r="21">
+      <x:c r="A21" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">6) Usa entre 2 y 5 días.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" t="inlineStr">
+    <x:row r="22">
+      <x:c r="A22" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">7) Guarda y pulsa "Importar" en la app.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" t="inlineStr">
+    <x:row r="23">
+      <x:c r="A23" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">8) TOP+BACK (opcional, columna H) = "sí": la 1.ª serie es la top</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" t="inlineStr">
+    <x:row r="24">
+      <x:c r="A24" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">   (fija la progresión) y el resto back-offs con el % menos de peso (I)</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" t="inlineStr">
+    <x:row r="25">
+      <x:c r="A25" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">   hasta el RIR de la columna J. Vacío o "no" = series rectas.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" t="inlineStr">
+    <x:row r="26">
+      <x:c r="A26" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">9) SUPERSERIE (columna K): pon el mismo número (1, 2…) en dos filas</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" t="inlineStr">
+    <x:row r="27">
+      <x:c r="A27" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">   seguidas para enlazarlas y alternar sus series sin descanso.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" t="inlineStr">
+    <x:row r="28">
+      <x:c r="A28" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">10) DROP SET (columna L) = "sí": tras la última serie, bajadas de peso</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" t="inlineStr">
+    <x:row r="29">
+      <x:c r="A29" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">    seguidas del % de la columna M, sin descanso.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" t="inlineStr">
+    <x:row r="30">
+      <x:c r="A30" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">11) Cada fila admite solo UNA modalidad: top+back, drop set o superserie;</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" t="inlineStr">
+    <x:row r="31">
+      <x:c r="A31" s="0" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">    el Excel bloquea las combinaciones y la app deshace las que lleguen.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FICHA DE LA RUTINA</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Rutina generada:</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B28" s="0" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Routine 10 - 2 days - MEV hypertrophy, 60 min max - men</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Objetivo:</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B29" s="0" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">General hypertrophy with minimum effective volume, sessions under 60 minutes, and exercises with quick setup.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Notas de diseño:</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B30" s="0" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Machines, cables, and stable movement patterns are prioritized to reduce specific warm-ups, equipment changes, and nonproductive fatigue.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Progresión recomendada:</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B31" s="0" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Double progression: when all sets reach the top of the range at the prescribed RIR, increase the load by the smallest possible amount and return to the bottom of the range.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Intensificadores:</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B32" s="0" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Superset = alternate the sets of the two linked exercises with no rest between them; drop set = after the last set, successive load drops with no rest. Each row allows only one method (top+back, superset or drop set). Day 1: superset Press en máquina convergente + Remo en máquina con apoyo de pecho; superset Extensión en cuerda en polea + Curl en cuerda en polea; drop set Elevación lateral en máquina (-20 %). Day 2: superset Press inclinado en máquina + Jalón al pecho agarre neutro cerrado; superset Gemelo en prensa + Crunch en máquina; drop set Curl femoral tumbado (-20 %).</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>